<commit_message>
vault backup: 2026-08-03 19:25:30
</commit_message>
<xml_diff>
--- a/Codex/projects/考研英语外刊精读/articles/Are stablecoins money/anki/anki.xlsx
+++ b/Codex/projects/考研英语外刊精读/articles/Are stablecoins money/anki/anki.xlsx
@@ -41,12 +41,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：In textbooks money is a means of exchange, a store of value and a unit of account. 译：在教科书里，货币是一种交换媒介、一种价值储藏手段，也是一种记账单位。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：交换媒介 / 价值储藏手段 / 记账单位。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：经济类说明文的定义三件套，常用于判断概念是否成立。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：means = method/function 方法或功能；store = a place or function for keeping value 储藏功能；unit = standard measure 标准单位；account = record/账目，不是账户登录。&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：account 可指账户、叙述、账目；这里 unit of account 是“记账单位”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：中性、定义性、学术语体。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：交换媒介 / 价值储藏手段 / 记账单位。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：In textbooks money is a means of exchange, a store of value and a unit of account.&lt;br&gt;译：在教科书里，货币是一种交换媒介、一种价值储藏手段，也是一种记账单位。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：这是 money 的三功能定义；account 在这里是“记账”，不是“账户”。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：经济类定义题会围绕这三点判断某物是否算 money。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Gold once served as a store of value. 译：黄金曾经充当价值储藏手段。&lt;br&gt;2. Language can be a means of cultural exchange. 译：语言可以成为文化交流的媒介。</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：作者先给出货币的教科书定义，再用稳定币逐项对照。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：细节题会问某事是否具备 money 的功能；选项常用 medium, measure, standard, record 替换。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Gold once served as a store of value in many societies. 译：黄金曾在许多社会中充当价值储藏手段。&lt;br&gt;Language can be a means of cultural exchange. 译：语言可以成为文化交流的媒介。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：可用于经济、文化、教育类作文：Reading is not only a means of acquiring knowledge, but also a store of cultural memory. 译：阅读不仅是获取知识的手段，也是文化记忆的储藏方式。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Reading is not only a means of acquiring knowledge, but also a store of cultural memory. 译：阅读不仅是获取知识的手段，也是文化记忆的储藏方式。</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -58,17 +58,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>a giant confidence trick</t>
+          <t>keep count with</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：In life it is a giant confidence trick: people trade with it, save it and keep count with it because everyone else does. 译：在现实生活中，货币是一场巨大的信任把戏：人们使用它，是因为其他人也使用它。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：巨大的信任把戏；靠共同信任维持的机制。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：熟词组合 + 诙谐表达。不是说货币真是骗局，而是强调社会信任。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：confidence = trust 信任；trick = device/deception 把戏或骗局。English: the phrase sounds witty and slightly ironic, because a serious institution is described like a magic trick.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：trick 可指技巧、窍门、恶作剧、骗局；这里偏“看似神奇但靠信任运转的机制”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：诙谐、轻微讽刺，但不是强烈贬义。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：用……计数 / 记账。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：People trade with it, save it and keep count with it because everyone else does.&lt;br&gt;译：人们用它交易、储蓄并计数，是因为其他人也这么做。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：count 是“计数”；keep count with money = 用货币来记录价值。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：翻译时不要译成“保持数量”，应译为“用……计数/记账”。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Calories help athletes keep count with daily energy intake. 译：热量帮助运动员记录每日能量摄入。&lt;br&gt;2. A clear budget helps a family keep count with its spending. 译：清晰预算帮助家庭记录支出。</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：作者用它概括货币的社会基础：大家都信，所以它能流通。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：态度题不要选 fraud/scam 这种过强贬义；更稳的是 public trust / shared belief。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Public credit is a confidence trick that depends on responsible institutions. 译：公共信用是一种依赖负责任制度的信任机制。&lt;br&gt;A classroom rule works only when it becomes a shared confidence trick among students. 译：课堂规则只有在学生共同相信并遵守时才会真正发挥作用。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：可用于诚信、社会责任、制度信任：A modern society depends on a confidence trick called public trust. 译：现代社会依赖一种名为公共信任的信任机制。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：不建议作文使用，语境较窄。</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -80,17 +80,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>keep count with</t>
+          <t>alloy / mere alloy</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：People trade with it, save it and keep count with it because everyone else does. 译：人们用它交易、储蓄并计数，是因为其他人也这么做。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：用……计数 / 记账。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：基础词 count 的短语义，放在经济语境中表示记录价值。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：keep = maintain/continue 保持；count = number or calculate 计数；with = using 借助。English: keep count with money means use money as the measuring tool.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：count 可作“数数、重要、有价值”；keep count 是“记录数量”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：中性、功能说明。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：合金；不过是金属合金。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Notes are just slips of paper; coins, mere alloy.&lt;br&gt;译：纸币不过是一张张纸；硬币也只是金属合金。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：alloy 是“合金”；mere = 只不过，用来降低表面价值。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：态度题中 mere 常暗示作者要看更深层原因。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. The medal was not mere alloy; it represented years of discipline. 译：那枚奖牌不只是合金，它代表多年的自律。&lt;br&gt;2. Coins are made from alloy rather than pure metal. 译：硬币由合金而非纯金属制成。</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：解释货币作为 unit of account 的现实作用。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：翻译题不要译成“保持数量”，要译成“用它计数/记账”。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：A company needs clear accounts to keep count with every project. 译：公司需要清楚的账目来记录每个项目。&lt;br&gt;Calories help athletes keep count with daily energy intake. 译：热量可以帮助运动员记录每日能量摄入。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Success is not mere luck; it is built on discipline. 译：成功不只是运气，而是建立在自律之上。</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -102,17 +102,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>mere alloy</t>
+          <t>liability</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Notes are just slips of paper; coins, mere alloy. 译：纸币不过是一张张纸；硬币也只是金属合金。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：不过是合金。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：mere 是考研态度词，表示“只不过、仅仅”，常降低事物表面价值。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：mere = only/nothing more than 仅仅；alloy = mixed metal 合金。English: the noun phrase omits coins are, making the sentence compact and literary.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：alloy 本义是合金；也可作动词表示“掺杂、削弱纯度”，如 joy alloyed with anxiety。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：轻描淡写，带一点反讽。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：负债；法律责任；不利因素。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Most money is simply data: some in the form of "reserves", liabilities of the central bank.&lt;br&gt;译：大多数货币只是数据，其中一部分以“准备金”形式存在，是中央银行的负债。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：liable = 有责任的；金融中 liability 常是“负债”，法律中是“责任”。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：不要见到 -ability 就当“能力”；金融语境优先译成“负债”。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Poor risk control became a serious liability for the firm. 译：糟糕的风险控制成了公司的严重隐患。&lt;br&gt;2. The hospital faced legal liability after the accident. 译：事故后医院面临法律责任。</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：作者说明货币实物本身没有神秘价值，价值来自制度信任。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：看到 mere + noun，作者往往在削弱表面意义，答案应找 deeper reason。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：The medal was not mere alloy; it represented years of discipline. 译：那枚奖牌不只是合金，它代表多年的自律。&lt;br&gt;Data are not mere numbers when they shape public policy. 译：当数据影响公共政策时，它们就不只是数字。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：可用于精神品质话题：Success is not mere luck; it is built on patience and discipline. 译：成功不只是运气，而是建立在耐心和自律之上。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：用户词表 alloy 已归入 mere alloy。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：A lack of honesty can turn talent into a liability. 译：缺乏诚信会让才能变成隐患。</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -124,17 +124,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>liability</t>
+          <t>at a keystroke</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Most money is simply data: some in the form of "reserves", liabilities of the central bank. 译：大多数货币只是数据，其中一部分以“准备金”形式存在，是中央银行的负债。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：负债；责任；不利因素。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：熟词僻义高频。法律和金融文章里 liability 常不是“能力”，而是“责任/负债”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：liable = legally responsible 有责任的；-ity = noun suffix 名词后缀。English: liability is something owed or a responsibility one must bear.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：1. 负债：bank liabilities 银行负债。2. 法律责任：legal liability 法律责任。3. 不利因素：His anger is a liability. 他的脾气是个隐患。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：正式、法律金融语体。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：敲一下键盘即可；通过一次电子操作。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Much more of it is created by banks calling loans and deposits into being at a keystroke.&lt;br&gt;译：更多货币则由银行敲一下键盘就创造出贷款和存款。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：key = 键；stroke = 一次按压。这个短语强调数字化操作很快。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：翻译题要联系 computer/data，不能译成“关键打击”。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. A payment can now be made at a keystroke. 译：现在一笔付款可以敲一下键盘完成。&lt;br&gt;2. Students can reach lectures at a keystroke. 译：学生轻点按键即可接触课程。</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：本文指央行准备金是中央银行负债。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：选项若把 liability 译成 ability/asset 通常是错；注意 asset 是资产，liability 是负债。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Poor risk control became a serious liability for the firm. 译：糟糕的风险控制成了公司的严重隐患。&lt;br&gt;The hospital faced legal liability after the accident. 译：事故后医院面临法律责任。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：可用于职场/社会责任：A lack of honesty can turn talent into a liability. 译：缺乏诚信会让才能变成隐患。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Public services are increasingly available at a keystroke. 译：公共服务越来越可以通过一次按键获得。</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -146,17 +146,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>at a keystroke</t>
+          <t>singleness</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Much more of it is created by banks calling loans and deposits into being at a keystroke. 译：更多货币则由银行敲一下键盘就创造出贷款和存款。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：敲一下键盘即可；非常迅速地通过电子操作完成。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：技术化表达，暗示现代金融创造货币的无形和高效。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：key = keyboard key 按键；stroke = hit/press 一击、一次按压。English: at a keystroke means with one simple computer action.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：stroke 可指击打、笔画、中风；keystroke 是电脑按键动作。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：轻松、现代、略带惊讶。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：统一性；同一货币在不同地方价值一致。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：First, singleness: a dollar in one bank is worth the same as one in another.&lt;br&gt;译：第一是统一性：一家银行中的一美元与另一家银行中的一美元价值相同。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：single = 单一/相同；-ness = 状态。这里不是“单身”，而是价值统一。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：本文核心标准：稳定币缺少 singleness，所以还不完全是货币。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. A national exam needs singleness of standards. 译：全国性考试需要标准统一。&lt;br&gt;2. Digital money requires singleness if users are to trust it. 译：数字货币若要获得信任，就需要价值统一性。</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：作者说明银行通过数据创造货币，而非铸造硬币。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：翻译时不要译成“在一次关键打击中”，应联系 computer/data。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：A payment can now be made at a keystroke. 译：现在一笔付款可以敲一下键盘完成。&lt;br&gt;Online learning allows students to reach lectures at a keystroke. 译：在线学习让学生轻点按键即可接触课程。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：科技生活作文可用：Public services are increasingly available at a keystroke. 译：公共服务越来越可以通过一次按键获得。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：The singleness of rules is essential to educational fairness. 译：规则统一对教育公平至关重要。</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -168,17 +168,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>singleness</t>
+          <t>frictionlessly</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：First, singleness: a dollar in one bank is worth the same as one in another. 译：第一是统一性：一家银行中的一美元与另一家银行中的一美元价值相同。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：统一性；不同形式的同一货币价值一致。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：本文核心判断标准。稳定币是否是 money，要看它是否具备 singleness。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：single = one/same 单一、相同；-ness = state 名词后缀。English: singleness here means the sameness of value across different holders or institutions.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：不是“单身状态”，而是金融语境中的“统一性/同一性”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：学术、概念化。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：无摩擦地；顺畅地。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Dollars move more or less frictionlessly between banks, people, businesses and governments.&lt;br&gt;译：美元可以在银行、个人、企业和政府之间大体上无摩擦地流动。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：friction 是“摩擦/阻力”；-less = 没有；这里指流程阻力小。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：阅读中常被 smoothly, efficiently, with little resistance 替换。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Information should move frictionlessly across departments. 译：信息应在部门之间顺畅流动。&lt;br&gt;2. A good app lets users pay frictionlessly. 译：好应用能让用户顺畅付款。</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：后文说 stablecoins lack singleness，因为价格偶尔偏离 1 美元。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：定义题定位词；看到 stablecoins lack singleness，应理解为价值不能完全无差别。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：A national exam needs singleness of standards across different provinces. 译：全国性考试需要各省标准统一。&lt;br&gt;Digital money requires singleness if users are to trust it. 译：数字货币若要获得用户信任，就需要价值统一性。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：社会公平作文可用：The singleness of rules is essential to educational fairness. 译：规则统一对教育公平至关重要。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Digital tools can help knowledge flow frictionlessly. 译：数字工具能帮助知识顺畅流动。</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -190,17 +190,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>frictionlessly</t>
+          <t>extend or rein in lending</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Dollars move more or less frictionlessly between banks, people, businesses and governments. 译：美元可以在银行、个人、企业和政府之间大体上无摩擦地流动。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：无摩擦地；顺畅地。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：熟词 friction 从物理“摩擦”转为制度/流程阻力。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：friction = resistance 阻力；-less = without 无；-ly = adverb 副词。English: frictionlessly means with little delay, cost or resistance.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：friction 可指物理摩擦，也可指人际矛盾、制度阻力、交易成本。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：中性偏积极，强调效率。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：扩大或收紧放贷。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Banks extend or rein in lending.&lt;br&gt;译：银行会扩大或收紧放贷。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：lend = 借出；lending = 放贷；rein in = 控制、收紧。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：完形常考 extend/rein in 的反义关系；lend 和 borrow 别混。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Banks may rein in lending when risks rise. 译：风险上升时，银行可能收紧放贷。&lt;br&gt;2. A bank can extend lending to small businesses. 译：银行可以向小企业扩大放贷。</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：说明传统美元体系的可转移性。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：阅读中常被替换为 smoothly, with little resistance, efficiently。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Good teamwork allows information to move frictionlessly across departments. 译：良好团队协作让信息在部门之间顺畅流动。&lt;br&gt;A well-designed app lets users pay frictionlessly. 译：设计良好的应用让用户顺畅付款。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：科技/职场作文可用：Digital tools can help knowledge flow frictionlessly. 译：数字工具能帮助知识顺畅流动。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Financial institutions should extend lending responsibly. 译：金融机构应负责任地扩大信贷。</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -212,17 +212,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>extend or rein in lending</t>
+          <t>the lender of last resort</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：The supply of money adjusts as required--usually quite calmly, as banks extend or rein in lending. 译：货币供应量会按需要调整，通常相当平稳，因为银行会扩大或收紧放贷。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：扩大或收紧放贷。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：lend 是基础词，但 lending 在经济文章中常指信贷投放。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：lend = give money temporarily 借出；lending = the activity of giving loans 放贷；rein in = control/limit 控制、收紧。English: extend lending expands credit; rein in lending restricts credit.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：lend 借出；borrow 借入。中文“借”容易双向混淆。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：中性政策表达。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：最后贷款人；危机中提供最终资金支持的机构。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：In a crisis, money pours forth from the central bank, the lender of last resort.&lt;br&gt;译：在危机中，资金会从中央银行这个最后贷款人那里大量涌出。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：last resort = 最后办法；lender of last resort 通常指央行。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：细节题可替换为 emergency backstop / central-bank support。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. The central bank acted as the lender of last resort. 译：央行充当最后贷款人。&lt;br&gt;2. Public hospitals often serve as providers of last resort. 译：公立医院常发挥最后兜底作用。</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：说明货币供给弹性如何由银行信贷调节。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：完形常考 extend/rein in 的反义关系；翻译要补出“放贷”。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Banks may rein in lending when the economy weakens. 译：经济走弱时，银行可能收紧放贷。&lt;br&gt;A school can extend support to students from poor families. 译：学校可以向贫困家庭学生扩大支持。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：经济作文可用：Financial institutions should extend lending responsibly rather than fuel reckless expansion. 译：金融机构应负责任地扩大信贷，而不是助长鲁莽扩张。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：用户词表 lend 已归入 extend or rein in lending。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Public institutions should serve as a last resort for vulnerable groups. 译：公共机构应为弱势群体提供最后保障。</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -234,17 +234,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>the lender of last resort</t>
+          <t>circumstances</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：In a crisis, money pours forth from the central bank, the lender of last resort. 译：在危机中，资金会从中央银行这个最后贷款人那里大量涌出。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：最后贷款人；危机中提供最终流动性支持的机构。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：金融危机和央行职能核心术语。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：lender = one who lends money 贷款方；last resort = final option 最后手段。English: the lender of last resort is the institution that provides emergency liquidity when others cannot.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：resort 可指度假地，也可指“求助办法”；last resort 是“最后办法”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：正式、制度性。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：情况；条件；环境。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：As circumstances change it adapts, for better or worse.&lt;br&gt;译：随着环境变化，它也会调整，结果可能变好，也可能变坏。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：常用复数 circumstances；under no circumstances = 绝不。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：阅读中常被 conditions, situation, context 替换。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Teaching methods should change as circumstances change. 译：教学方法应随着情况变化而调整。&lt;br&gt;2. Under difficult circumstances, honesty becomes even more valuable. 译：在困难情况下，诚实更加可贵。</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：作者用它解释传统货币体系在危机中为何有弹性。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：细节题会把它替换为 emergency backstop / central-bank support。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：The central bank acted as the lender of last resort during the banking panic. 译：银行恐慌期间，央行充当最后贷款人。&lt;br&gt;In public health, government hospitals often become providers of last resort. 译：在公共卫生领域，公立医院常成为最后兜底者。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：社会责任作文可迁移 last resort：Public institutions should serve as a last resort for vulnerable groups. 译：公共机构应为弱势群体提供最后保障。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：As circumstances change, public policies should adapt responsibly. 译：随着情况变化，公共政策应负责任地调整。</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -256,17 +256,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>as circumstances change</t>
+          <t>a giddying lot of changes</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：As circumstances change it adapts, for better or worse. 译：随着环境变化，它也会调整，结果可能变好，也可能变坏。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：随着情况变化。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：circumstance 是考研高频抽象名词，常用于环境、条件、背景。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：circum = around 周围；stance = standing 状态。English: circumstances are surrounding conditions that affect a decision or event.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：常用复数 circumstances 表“情况/条件”；under no circumstances = 绝不。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：中性、背景条件。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：一大堆令人目眩的变化。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Digital innovations--a giddying lot of changes if ever there was one--pose an awkward question.&lt;br&gt;译：数字创新带来一大堆令人目眩的变化，并提出了一个棘手问题。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：giddy = 头晕/兴奋；giddying 修饰变化时表示快而复杂。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：态度题别选单纯赞美；这里强调变化密集、监管复杂。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Online platforms have brought a giddying lot of changes to education. 译：在线平台给教育带来了大量令人目眩的变化。&lt;br&gt;2. Remote work created a giddying lot of changes in offices. 译：远程办公给职场带来大量变化。</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：作者说明货币制度会随技术和环境变化而调整。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：选项常用 conditions, situation, context 替换。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Teaching methods should change as circumstances change. 译：教学方法应随着情况变化而调整。&lt;br&gt;Under difficult circumstances, honesty becomes even more valuable. 译：在困难情况下，诚实更加可贵。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：作文万能句：As circumstances change, public policies should adapt in a responsible way. 译：随着情况变化，公共政策应负责任地调整。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Artificial intelligence has brought a giddying lot of changes to modern life. 译：人工智能给现代生活带来了大量令人目眩的变化。</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -278,17 +278,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>a giddying lot of changes</t>
+          <t>be in charge of</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Digital innovations--a giddying lot of changes if ever there was one--pose an awkward question. 译：数字创新带来一大堆令人目眩的变化，并提出了一个棘手问题。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：一大堆令人目眩的变化。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：giddying 是外刊态度词，表示变化快到让人眩晕。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：giddy = dizzy/excited 眩晕的、兴奋的；a lot of = many 大量。English: giddying suggests speed, confusion and excitement at the same time.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：giddy 可指头晕，也可指轻浮兴奋；giddying 修饰变化时指“令人眼花缭乱”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：轻微夸张，带外刊诙谐。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：负责；掌管。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Digital innovations pose an awkward question to those in charge of the arrangement.&lt;br&gt;译：数字创新给负责这套安排的人提出了一个棘手问题。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：charge 有“费用、指控、充电、负责”；in charge of = responsible for。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：翻译时结合语境判断，不要误译为“收费”。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Teachers in charge of online classes need clear rules. 译：负责网课的教师需要明确规则。&lt;br&gt;2. People in charge of public funds must act transparently. 译：负责公共资金的人必须透明行事。</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：作者评价数字创新变化密集，监管难度上升。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：态度题要识别作者不是单纯赞美，而是强调复杂性。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：The rise of online platforms has brought a giddying lot of changes to education. 译：在线平台兴起给教育带来了大量令人目眩的变化。&lt;br&gt;The workplace has faced a giddying lot of changes since remote work became common. 译：远程办公普及以来，职场经历了大量令人眼花缭乱的变化。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：科技作文可用：Artificial intelligence has brought a giddying lot of changes to modern life. 译：人工智能给现代生活带来了大量令人目眩的变化。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Those in charge of companies should balance profit with social responsibility. 译：企业负责人应平衡利润与社会责任。</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -300,17 +300,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>be in charge of</t>
+          <t>chew over</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Digital innovations pose an awkward question to those in charge of the arrangement. 译：数字创新给负责这套安排的人提出了一个棘手问题。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：负责；掌管。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：基础短语但写作和阅读高频，常作后置定语。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：charge = responsibility/control 责任、掌管；in charge of = responsible for 负责。English: those in charge of means the people responsible for managing something.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：charge 可指费用、指控、充电、负责；本文是负责。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：中性、管理语境。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：仔细琢磨；反复讨论。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Stablecoins are an example chewed over in the CEPR report.&lt;br&gt;译：稳定币是 CEPR 报告中反复讨论的一个例子。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：chew 本义“咀嚼”；chew over = 像咀嚼一样反复思考。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：同义替换：consider, discuss, examine, think through。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. The committee chewed over the reform plan for weeks. 译：委员会反复讨论改革方案数周。&lt;br&gt;2. Students should chew over difficult passages before checking the translation. 译：学生应先琢磨难段，再看翻译。</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：指政策制定者和监管者。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：翻译时不要译成“收费的人”；结合 arrangement 判断为负责人。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Teachers in charge of online classes need clear rules. 译：负责网课的教师需要明确规则。&lt;br&gt;People in charge of public funds must act transparently. 译：负责公共资金的人必须透明行事。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：职场作文可用：Those in charge of companies should balance profit with social responsibility. 译：企业负责人应平衡利润与社会责任。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Young people should chew over complex information instead of accepting it blindly. 译：年轻人应仔细思考复杂信息，而不是盲目接受。</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -322,17 +322,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>chew over</t>
+          <t>the sole subject of</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Stablecoins are an example chewed over in the CEPR report. 译：稳定币是 CEPR 报告中反复讨论的一个例子。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：仔细琢磨；反复讨论。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：动词短语，外刊常用口语化表达。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：chew = bite food 咀嚼；chew over = think about or discuss carefully 反复思考/讨论。English: it turns mental processing into the image of chewing food.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：chew 本义咀嚼；短语 chew over 是抽象义。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：口语化、形象。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：……的唯一主题。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Stablecoins are the sole subject of another new study, by the Bank for International Settlements.&lt;br&gt;译：稳定币也是国际清算银行另一项新研究的唯一主题。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：sole = only；subject = 主题。sole 比 main 更绝对。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：细节题注意 sole 的绝对程度，不能偷换成“主要之一”。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Mental health became the sole subject of the meeting. 译：心理健康成了会议的唯一主题。&lt;br&gt;2. Food safety was the sole subject of the report. 译：食品安全是这份报告的唯一主题。</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：说明稳定币已被经济学报告深入讨论。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：同义替换：consider, discuss, examine, think through。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：The committee chewed over the reform plan for weeks. 译：委员会反复讨论改革方案数周。&lt;br&gt;Students should chew over difficult passages before checking the translation. 译：学生应先琢磨难段，再看翻译。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：学习方法作文可用：Young people should chew over complex information instead of accepting it blindly. 译：年轻人应仔细思考复杂信息，而不是盲目接受。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Environmental protection should not be the sole subject of governments. 译：环境保护不应只是政府的议题。</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -344,17 +344,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>the sole subject of</t>
+          <t>be pegged to fiat currencies</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Stablecoins are the sole subject of another new study, by the Bank for International Settlements. 译：稳定币也是国际清算银行另一项新研究的唯一主题。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：……的唯一主题。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：sole 是考研高频形容词，表示唯一的、单独的。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：sole = only/single 唯一的；subject = topic 主题。English: the sole subject of a study means the study focuses only on that topic.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：subject 可指主题、科目、臣民、受试者；这里是研究主题。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：正式、中性。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：锚定法定货币。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Of those pegged to fiat currencies, 99.4% by value are tied to the dollar.&lt;br&gt;译：在那些锚定法定货币的稳定币中，按价值计算有 99.4% 与美元挂钩。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：peg = 固定/挂钩；fiat currency = 政府法定货币。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：细节题常用 fixed to, linked to, tied to 替换 pegged to。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Some currencies are pegged to the dollar. 译：一些货币与美元挂钩。&lt;br&gt;2. A school's budget may be pegged to student numbers. 译：学校预算可能与学生人数挂钩。</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：强调稳定币已成为独立研究对象。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：选项可替换为 exclusive focus / main focus, 但 sole 比 main 更绝对。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Mental health became the sole subject of the school meeting. 译：心理健康成了学校会议的唯一主题。&lt;br&gt;Food safety was the sole subject of the public report. 译：食品安全是这份公共报告的唯一主题。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：作文可用：Environmental protection should not be the sole subject of governments; it also requires individual action. 译：环境保护不应只是政府的议题，也需要个人行动。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：不建议作文使用，语境较窄。</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -366,17 +366,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>be pegged to fiat currencies</t>
+          <t>Treasury bills / reverse repos</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Of those pegged to fiat currencies, 99.4% by value are tied to the dollar. 译：在那些锚定法定货币的稳定币中，按价值计算有 99.4% 与美元挂钩。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：锚定法定货币。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：peg 和 fiat 都是金融科技文章高价值词。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：peg = fix or attach 固定、挂钩；fiat = official order 官方命令；fiat currency = money declared legal by a government 法定货币。English: pegged to means fixed against a reference value.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：peg 本义木钉/钉住；金融中指汇率或价格挂钩。fiat 不是菲亚特汽车，而是政府法令。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：正式、金融语体。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：美国短期国库券 / 逆回购。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Dollar stablecoins are backed mainly by Treasury bills, reverse repos and bank deposits.&lt;br&gt;译：美元稳定币主要由美国短期国库券、逆回购和银行存款支撑。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：这两个都属于稳定币储备资产；理解为 safe short-term financial assets 即可。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：考研阅读只需知道它们是支撑资产，不必深挖金融计算。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Treasury bills are short-term government debt. 译：短期国库券是短期政府债务。&lt;br&gt;2. Reverse repos are often used in short-term money markets. 译：逆回购常用于短期货币市场。</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：说明绝大多数稳定币与美元等法币挂钩。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：细节题可能用 fixed to, linked to, tied to 替换 pegged to。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Some currencies are pegged to the dollar to reduce exchange-rate volatility. 译：一些货币与美元挂钩以减少汇率波动。&lt;br&gt;A school's budget may be pegged to student numbers. 译：学校预算可能与学生人数挂钩。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：不建议作文使用，语境较窄。</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -388,17 +388,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>be backed by Treasury bills and reverse repos</t>
+          <t>be backed by</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Dollar stablecoins are backed mainly by Treasury bills, reverse repos and bank deposits. 译：美元稳定币主要由美国短期国库券、逆回购和银行存款支撑。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：由短期国库券、逆回购等资产支撑。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：be backed by 是核心，Treasury bills 与 reverse repos 理解金融支撑资产。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：back = support 支持；backed by = supported/secured by 由……支持或担保；Treasury bills = short-term government debt 短期国债；reverse repo = secured short-term lending arrangement 逆回购。&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：back 可指背部、支持、资助、作担保；本文是资产支撑。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：正式、金融语体。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：由……支撑；由……支持。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Dollar stablecoins are backed mainly by Treasury bills, reverse repos and bank deposits.&lt;br&gt;译：美元稳定币主要由美国短期国库券、逆回购和银行存款支撑。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：back 作动词不是“后背”，而是 support。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：翻译题常译为“由……支撑/担保/支持”。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. The scholarship programme is backed by local companies. 译：该奖学金项目由当地企业支持。&lt;br&gt;2. Public promises must be backed by practical action. 译：公共承诺必须由实际行动支撑。</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：解释稳定币背后储备资产来源。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：翻译题要译成“由……支撑/担保”，不要译成“被……背着”。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：The scholarship programme is backed by local companies. 译：该奖学金项目由当地企业支持。&lt;br&gt;The payment system is backed by short-term safe assets. 译：该支付系统由短期安全资产支撑。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：社会责任作文可用：Public promises must be backed by practical action. 译：公共承诺必须由实际行动支撑。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：用户词表 Treasury bills、reverse repos、be backed 已合并为一张高价值词组卡。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Educational fairness should be backed by sustained investment. 译：教育公平应由持续投入支撑。</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -415,12 +415,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：They are still mainly used for trading crypto assets. 译：它们目前仍主要用于交易加密资产。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：加密资产。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：科技金融热点词，阅读中不必深挖技术，但要知道它指数字加密资产。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：crypto = hidden/encrypted 加密的；asset = something valuable 资产。English: crypto assets are digital assets secured by cryptographic technology.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：asset 是资产，不是优势 advantage；crypto 可作 cryptocurrency 的缩写。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：中性、技术经济语体。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：加密资产。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：They are still mainly used for trading crypto assets.&lt;br&gt;译：它们目前仍主要用于交易加密资产。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：crypto = 加密；asset = 资产。别把 asset 译成 advantage。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：范围题注意：crypto assets 不等于所有 digital payments。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Regulators worry that crypto assets may create new risks. 译：监管者担心加密资产可能带来新风险。&lt;br&gt;2. Young investors should understand crypto assets before buying them. 译：年轻投资者购买加密资产前应先了解它们。</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：说明稳定币目前主要用途仍在加密货币交易。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：选项若把 crypto assets 泛化成 all digital payments，范围扩大。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Regulators worry that crypto assets may create new financial risks. 译：监管者担心加密资产可能带来新的金融风险。&lt;br&gt;Young investors should understand the risks of crypto assets before buying them. 译：年轻投资者购买加密资产前应了解其风险。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：不建议作文使用，语境较窄。</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -437,12 +437,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Stablecoins can make payments slicker and financial intermediation more competitive. 译：稳定币可以让支付更顺畅，让金融中介更具竞争性。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：金融中介；资金供需之间的撮合服务。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：intermediation 是抽象名词，经济阅读高频。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：inter- = between 在……之间；mediate = connect or intervene 调解/居中连接；-ion = noun 名词后缀。English: financial intermediation links savers, borrowers and payment users.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：mediate 可指调解，也可指在中间起作用；intermediary 是中介者。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：正式、学术。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：金融中介；连接储蓄者、借款者和支付用户的服务。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Stablecoins can make payments slicker and financial intermediation more competitive.&lt;br&gt;译：稳定币可以让支付更顺畅，让金融中介更具竞争性。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：inter- = between；mediate = 居中连接；合起来就是“在中间撮合”。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：经济类阅读中可替换为 financial services between parties。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Banks play a key role in financial intermediation. 译：银行在金融中介中发挥关键作用。&lt;br&gt;2. Digital platforms are changing financial intermediation. 译：数字平台正在改变金融中介服务。</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：说明稳定币可能提高金融服务竞争。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：阅读中可替换为 financial services between parties / middleman function。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Banks play a key role in financial intermediation. 译：银行在金融中介中发挥关键作用。&lt;br&gt;Digital platforms are changing financial intermediation for small businesses. 译：数字平台正在改变小企业的金融中介服务。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：经济作文可用：Technology can make financial intermediation more inclusive. 译：技术可以让金融中介服务更具包容性。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Technology can make financial intermediation more inclusive. 译：技术可以让金融中介服务更具包容性。</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -459,12 +459,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Combined with smart contracts, they can also speed up settlements and payments, obviating the need to go through a long chain of lawyers and banks. 译：与智能合约结合后，它们还能加快结算和付款，从而免去经过一长串律师和银行的需要。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：消除做某事的必要。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：高级动词，翻译和作文都很有价值。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：obviate = remove/prevent the need 消除必要性；the need to do = 做某事的需要。English: obviate is formal and often used for systems that make an old step unnecessary.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：不要把 obviate 误解为 obvious；它是“排除、消除”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：正式、书面。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：消除做某事的必要；使某步骤不再需要。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Combined with smart contracts, they can also speed up settlements and payments, obviating the need to go through a long chain of lawyers and banks.&lt;br&gt;译：与智能合约结合后，它们还能加快结算和付款，从而免去经过一长串律师和银行的需要。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：obviate = remove the need；固定搭配 `obviate the need to do`。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：翻译题常译为“免去……的需要 / 使……不再必要”。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Online registration can obviate the need to wait in long lines. 译：在线注册可以免去长时间排队的需要。&lt;br&gt;2. Clear rules can obviate the need for repeated negotiation. 译：明确规则可以免去反复协商的需要。</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：说明稳定币与智能合约可以减少中间环节。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：翻译时常译为“使……不再必要 / 免去……需要”。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Online registration obviates the need to queue for hours. 译：在线注册免去了排队数小时的需要。&lt;br&gt;Clear rules can obviate the need for repeated negotiation. 译：明确规则可以免去反复协商的需要。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：科技作文可用：Digital public services can obviate the need for unnecessary paperwork. 译：数字公共服务可以免去不必要的文书手续。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Digital public services can obviate the need for unnecessary paperwork. 译：数字公共服务可以免去不必要的文书手续。</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -481,12 +481,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Stablecoins may find it hard to meet redemptions in a hurry without access to central-bank support. 译：如果没有中央银行支持，稳定币可能很难在紧急情况下满足赎回需求。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：满足赎回要求。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：金融风险核心搭配，meet 不是“见面”，而是“满足”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：meet = satisfy/fulfil 满足；redemption = repayment or exchange for value 赎回。English: meet redemptions means have enough money to pay people who want to cash out.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：redemption 可指赎回、救赎；金融中指把投资/票据换回现金。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：正式、风险语境。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：满足赎回要求。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Stablecoins may find it hard to meet redemptions in a hurry without access to central-bank support.&lt;br&gt;译：如果没有中央银行支持，稳定币可能很难在紧急情况下满足赎回需求。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：meet 在这里不是“见面”，而是 satisfy/fulfil；redemption = 赎回。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：熟词僻义：meet demand / meet requirements / meet redemptions。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. The fund sold assets to meet redemptions. 译：该基金出售资产以满足赎回要求。&lt;br&gt;2. Schools need enough teachers to meet students' needs. 译：学校需要足够教师来满足学生需求。</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：作者用它质疑稳定币缺少央行支持时的弹性。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：熟词 meet 高频考：meet demand / meet requirements / meet obligations。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：The fund sold assets to meet redemptions. 译：该基金出售资产以满足赎回要求。&lt;br&gt;Schools need enough teachers to meet students' needs. 译：学校需要足够教师来满足学生需求。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：可迁移 meet needs：Public policy should meet citizens' basic needs before pursuing efficiency. 译：公共政策应先满足公民基本需求，再追求效率。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Public policy should meet citizens' basic needs before pursuing efficiency. 译：公共政策应先满足公民基本需求，再追求效率。</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -503,12 +503,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：The BIS notes that stablecoins account for a fair bit of illicit activity on blockchains. 译：国际清算银行指出，稳定币在区块链上的非法活动中占有相当一部分。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：非法活动。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：illicit 是态度鲜明的负面词，常用于法律、道德、监管文章。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：il- = not 否定前缀；licit = lawful 合法的。English: illicit means illegal or forbidden by rules.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：illegal 更普通；illicit 更正式，常带道德或监管意味。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：负面、正式。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：非法活动。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Stablecoins account for a fair bit of illicit activity on blockchains.&lt;br&gt;译：稳定币在区块链上的非法活动中占有相当一部分。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：il- 是否定前缀；licit = lawful 合法的；illicit = illegal。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：态度题中 illicit 明确指负面风险。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. The city cracked down on illicit trade near schools. 译：该市打击学校附近的非法交易。&lt;br&gt;2. Platforms must prevent illicit activity without harming normal users. 译：平台必须防止非法活动，同时不伤害正常用户。</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：说明稳定币带来的监管风险。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：态度题中 illicit 几乎必然指向 negative risk。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：The city cracked down on illicit trade near schools. 译：该市打击学校附近的非法交易。&lt;br&gt;Online platforms must prevent illicit activity without harming normal users. 译：网络平台必须防止非法活动，同时不伤害正常用户。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：社会责任作文可用：Technology firms should prevent illicit activity on their platforms. 译：科技公司应防止其平台上的非法活动。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Technology firms should prevent illicit activity on their platforms. 译：科技公司应防止其平台上的非法活动。</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -525,12 +525,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：A recent report suggests the biggest culprit is a rouble stablecoin. 译：最近一份报告显示，最大的罪魁祸首是一种卢布稳定币。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：卢布稳定币。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：这是具体案例，不是高频必背词；但用户已摘录，可作为 topic term 理解。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：rouble/ruble = Russia's currency 卢布；stablecoin = digital currency pegged to an asset 稳定币。English: the phrase identifies a specific type of stablecoin linked to roubles.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：rouble 是货币名；不必扩展为政治立场，只理解为案例。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：中性词组，但出现在 illicit activity 语境中带负面背景。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：卢布稳定币。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：A recent report by Chainalysis suggests the biggest culprit is a rouble stablecoin.&lt;br&gt;译：Chainalysis 最近的一份报告显示，最大的罪魁祸首是一种卢布稳定币。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：rouble/ruble = 俄罗斯卢布；这是原文具体例子，理解即可。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：细节题只定位它是 culprit，不要泛化成所有稳定币。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. The report identified a rouble stablecoin as a specific risk. 译：报告把一种卢布稳定币识别为具体风险。&lt;br&gt;2. A stablecoin may be linked to a national currency. 译：稳定币可能与某种国家货币挂钩。</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：用于说明非法活动中最大问题来源。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：细节题只需知道它是 culprit 的具体例子，不要泛化成 all stablecoins。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：A rouble stablecoin may be used where access to dollars is limited. 译：在美元获取受限的地方，卢布稳定币可能被使用。&lt;br&gt;The report treated the rouble stablecoin as a specific risk, not as the whole market. 译：报告把卢布稳定币视为一个具体风险，而不是整个市场。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：理解即可，不建议迁移到作文。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：不建议作文使用，语境较窄。</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -547,12 +547,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：A recent report by Chainalysis suggests the biggest culprit is a rouble stablecoin. 译：Chainalysis 最近的一份报告显示，最大的罪魁祸首是一种卢布稳定币。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：罪魁祸首；问题根源。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：可指人，也可指造成问题的事物，考研阅读常用于原因定位。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：culprit = person or thing responsible for a problem 责任者/原因。English: it often names the source of harm after evidence is presented.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：不只指罪犯，也可指抽象原因，如 pollution's culprit。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：负面、归因。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：罪魁祸首；问题根源。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：A recent report by Chainalysis suggests the biggest culprit is a rouble stablecoin.&lt;br&gt;译：Chainalysis 最近的一份报告显示，最大的罪魁祸首是一种卢布稳定币。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：culprit 可指人，也可指造成问题的事物。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：原因题看到 culprit，后面常是答案定位点。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Poor planning was the main culprit behind the failure. 译：规划不善是失败的主要原因。&lt;br&gt;2. Excessive screen time is often a culprit in poor sleep. 译：过度使用屏幕常是睡眠不佳的原因。</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：本文指出非法活动中最大问题来源。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：原因题看到 culprit，后面常是答案定位点。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Poor planning was the main culprit behind the project's failure. 译：规划不善是项目失败的主要原因。&lt;br&gt;Excessive screen time is often blamed as a culprit in poor sleep. 译：过度使用屏幕常被认为是睡眠不佳的一个原因。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：健康/教育作文可用：The real culprit is not technology itself, but the careless way people use it. 译：真正的问题根源不是技术本身，而是人们草率使用技术的方式。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：The real culprit is not technology itself, but careless use. 译：真正的问题根源不是技术本身，而是草率使用。</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -569,12 +569,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：They lose seigniorage, the difference between the value of money and the negligible cost of creating it. 译：它们会失去铸币税收益，也就是货币价值与创造货币的微不足道成本之间的差额。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：铸币税收益；发行货币所得收益。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：专业词，考研不要求拼写高频，但文章理解很关键。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：seigniorage historically comes from the lord's right to coin money. English: in modern economics, it means the profit a monetary authority earns by issuing money.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：不要译为普通 tax；它是发行货币带来的收益。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：正式、专业。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：铸币税收益；发行货币所得收益。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：They lose seigniorage, the difference between the value of money and the negligible cost of creating it.&lt;br&gt;译：它们会失去铸币税收益，即货币价值与创造货币的微不足道成本之间的差额。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：专业词。记成：造钱成本低，但钱有面值，中间差额就是 seigniorage。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：理解概念即可；翻译可括注“铸币收益”。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Central banks may lose seigniorage when private money spreads. 译：私人货币扩散时，央行可能失去铸币税收益。&lt;br&gt;2. Seigniorage matters because money is cheap to create but valuable to hold. 译：铸币税重要，因为货币创造成本低但持有价值高。</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：说明美元稳定币可能削弱央行收益和主权货币能力。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：翻译时可括注“铸币收益”，无需深挖公式。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Central banks may lose seigniorage when private digital currencies become popular. 译：私人数字货币普及时，央行可能失去铸币税收益。&lt;br&gt;Seigniorage matters because money is cheap to create but valuable to hold. 译：铸币税重要，因为货币创造成本低但持有价值高。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：理解概念即可，不做作文模板。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：不建议作文使用，语境较窄。</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -591,12 +591,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：They lose seigniorage, the difference between the value of money and the negligible cost of creating it. 译：它们会失去铸币税收益，即货币价值与创造货币的微不足道成本之间的差额。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：微不足道的；可忽略不计的。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：考研高频形容词，常修饰 cost, effect, risk, difference。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：neglect = ignore 忽视；-ible = able to be 可被……的。English: negligible means so small that it can almost be ignored.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：negligent = 疏忽的；negligible = 微不足道的，注意区分。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：正式、中性偏低估。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：微不足道的；可忽略不计的。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：They lose seigniorage, the difference between the value of money and the negligible cost of creating it.&lt;br&gt;译：它们会失去铸币税收益，即货币价值与创造货币的微不足道成本之间的差额。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：neglect = 忽视；negligible = 小到可以忽略。注意 negligent = 疏忽的。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：同义替换：minor, tiny, insignificant, marginal。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. The cost of sending an email is negligible. 译：发送电子邮件的成本微乎其微。&lt;br&gt;2. One plastic bag may seem negligible, but the total damage is large. 译：一个塑料袋似乎微不足道，但总体伤害很大。</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：说明造币成本相对货币面值极低。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：同义替换：minor, tiny, insignificant, marginal。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：The cost of sending an email is negligible. 译：发送电子邮件的成本微乎其微。&lt;br&gt;The effect of one plastic bag may seem negligible, but the total damage is large. 译：一个塑料袋的影响似乎微不足道，但总体伤害很大。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：环境作文可用：No individual effort is negligible when environmental protection becomes a shared duty. 译：当环保成为共同责任时，没有任何个人努力是微不足道的。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：No individual effort is negligible in environmental protection. 译：在环保中，任何个人努力都不是微不足道的。</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -608,17 +608,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>bond; be fond of</t>
+          <t>bond / be fond of</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：For governments, stablecoins are a helpful extra source of demand for their bonds. 译：对政府来说，稳定币是其债券需求的一个有用补充来源。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：bond = 债券；纽带。fond = 喜爱的。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：易混词辨析。本文 bond 是金融债券，不是关系纽带；fond 不在原文中，作为拼写/意义干扰。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：bond = financial debt security 债券, or connection 纽带；fond = liking something 喜爱的。English: one letter changes the word family completely.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：bond: government bonds 政府债券；social bonds 社会纽带。fond: be fond of reading 喜爱阅读。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：bond 金融语境正式；fond 日常情感色彩。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：bond = 债券；纽带。fond = 喜爱的。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Stablecoins are a helpful extra source of demand for their bonds.&lt;br&gt;译：稳定币是政府债券需求的一个有用补充来源。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：bond 和 fond 只差一个字母；本文 bond 是政府债券，不是 be fond of。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：金融语境 bond 常对应 debt/security；fond 对应 like/enjoy。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Many pension funds buy government bonds. 译：许多养老基金购买政府债券。&lt;br&gt;2. She is fond of reading serious magazines. 译：她喜欢阅读严肃杂志。</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：本文指政府债券需求，不是情感纽带。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：选项若出现 debt, Treasuries, securities 对应 bond；若出现 like/enjoy 才对应 fond。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Many pension funds buy government bonds. 译：许多养老基金购买政府债券。&lt;br&gt;She is fond of reading serious magazines. 译：她喜欢阅读严肃杂志。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：作文可用 bond 的抽象义：Shared responsibility can strengthen the bond between individuals and society. 译：共同责任能加强个人与社会之间的纽带。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Shared responsibility can strengthen the bond between individuals and society. 译：共同责任能加强个人与社会之间的纽带。</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -630,17 +630,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>amid a flurry of laws and proposals</t>
+          <t>amid a flurry of</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Amid the recent flurry of laws and proposals from the world's policymakers, there are some similarities. 译：在世界各国政策制定者最近密集出台法律和提案的浪潮中，可以看到一些共同点。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：在一连串/一阵密集的法律和提案中。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：flurry 是外刊常用词，表示短时间密集出现的一阵活动。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：amid = in the middle of 在……之中；flurry = sudden burst 一阵、纷纷出现。English: a flurry of laws suggests many policy moves arriving quickly.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：flurry 可指一阵雪、一阵忙乱、一连串行动。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：动态、新闻感。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：在一阵 / 一连串密集的……之中。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Amid the recent flurry of laws and proposals from the world's policymakers, there are some similarities.&lt;br&gt;译：在世界各国政策制定者最近密集出台法律和提案的浪潮中，可以看到一些共同点。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：amid = 在……之中；flurry = 一阵密集活动。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：常作背景开头，暗示事情短时间大量出现。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Amid a flurry of reforms, schools need clear priorities. 译：在一连串改革中，学校需要明确优先事项。&lt;br&gt;2. The firm hired more engineers amid a flurry of new orders. 译：在新订单纷至沓来之际，公司招聘了更多工程师。</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：转入各国监管稳定币的政策浪潮。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：背景句中 amid 常引出大环境；flurry 常暗示速度快、数量多。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Amid a flurry of reforms, schools need clear priorities. 译：在一连串改革中，学校需要明确优先事项。&lt;br&gt;The firm hired more engineers amid a flurry of new orders. 译：在新订单纷至沓来之际，公司招聘了更多工程师。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：作文开头可用：Amid a flurry of technological changes, society must protect both efficiency and fairness. 译：在技术变化纷至沓来之际，社会必须同时保护效率与公平。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Amid a flurry of technological changes, society must protect fairness. 译：在技术变化纷至沓来之际，社会必须保护公平。</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -657,12 +657,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：All require redemption at par, but some are vague about how quick it should be. 译：所有规则都要求按面值赎回，但有些规则对赎回速度应有多快仍表述模糊。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：按面值赎回。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：at par 是金融固定搭配，par 指票面价值/面值。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：redemption = cashing out/reclaiming value 赎回；par = face value 面值。English: redemption at par means one unit can be redeemed for its stated value.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：par 可指标准水平，如 below par 状态不佳；金融中是面值。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：正式、金融监管语境。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：按面值赎回。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：All require redemption at par, but some are vague about how quick it should be.&lt;br&gt;译：所有规则都要求按面值赎回，但有些规则对赎回速度应有多快仍表述模糊。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：par = face value 面值；at par = 按面值。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：细节题可能替换成 get back face value。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. The fund promised redemption at par. 译：该基金承诺按面值赎回。&lt;br&gt;2. Some gift cards cannot be redeemed at par after fees are deducted. 译：扣除费用后，有些礼品卡无法按面值兑换。</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：各国稳定币规则的共同要求。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：细节题可能问 stablecoin holders can get back face value。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：The fund promised redemption at par during normal market conditions. 译：该基金承诺在正常市场条件下按面值赎回。&lt;br&gt;Some gift cards cannot be redeemed at par after fees are deducted. 译：扣除费用后，有些礼品卡无法按面值兑换。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：不建议作文使用，语境较窄。</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -679,12 +679,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：All require redemption at par, but some are vague about how quick it should be. 译：所有规则都要求按面值赎回，但有些规则对速度多快仍表述模糊。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：对……含糊；没有说清楚。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：vague 是考研高频态度词，常表示批评规则、观点或解释不清。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：vague = unclear/not specific 模糊的；about = concerning 关于。English: be vague about means fail to give precise details.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：vague 可形容记忆、说法、计划、规则；vaguely 是副词。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：批评、负面。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：对……含糊；没有说清楚。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：All require redemption at par, but some are vague about how quick it should be.&lt;br&gt;译：所有规则都要求按面值赎回，但有些规则对速度多快仍表述模糊。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：vague = unclear/not specific；常用于批评规则、计划、说法不清。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：态度题中 vague 指向 insufficient clarity。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. The policy is vague about who will pay the cost. 译：该政策没有说清谁来承担成本。&lt;br&gt;2. His career plan remained vague after graduation. 译：毕业后他的职业规划仍然模糊。</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：作者指出监管规则仍有不明确处。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：态度题中 vague 指向 insufficient clarity，而不是 neutral。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：The policy is vague about who will pay the cost. 译：该政策没有说清谁来承担成本。&lt;br&gt;His career plan remained vague after graduation. 译：毕业后他的职业规划仍然模糊。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：作文可用：Rules should not be vague about responsibility. 译：规则不应在责任问题上含糊不清。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Rules should not be vague about responsibility. 译：规则不应在责任问题上含糊不清。</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -701,12 +701,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：The Bank of England has proposed 30% be in deposits at the central bank and 70% in short-term gilts. 译：英格兰银行提议 30% 存放在央行，70% 投资于短期英国国债。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：短期英国国债。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：gilt 是英国金融语境下的政府债券，理解即可。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：gilt = UK government bond 英国国债；short-term = maturing soon 短期的。English: gilts are generally viewed as safe sovereign debt.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：gilt 也可指镀金；金融中指英国政府债券。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：正式、英国金融语境。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：短期英国国债。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：The Bank of England has proposed 30% be in deposits at the central bank and 70% in short-term gilts.&lt;br&gt;译：英格兰银行提议 30% 存放在央行，70% 投资于短期英国国债。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：gilt 在英国金融语境中指 government bond；理解成英国国债即可。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：阅读中不必深挖，只需知道它是安全短期资产。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Pension funds often hold gilts for stability. 译：养老基金常持有英国国债以保持稳定。&lt;br&gt;2. Short-term government bonds are usually safer than risky corporate debt. 译：短期政府债券通常比高风险公司债更安全。</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：说明英国监管要求稳定币储备放入安全短期资产。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：阅读中可理解为 government bonds，不必纠结术语。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Pension funds often hold gilts for stability. 译：养老基金常持有英国国债以保持稳定。&lt;br&gt;Short-term government bonds are usually safer than risky corporate debt. 译：短期政府债券通常比高风险公司债更安全。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：不建议作文使用，语境较窄。</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -723,12 +723,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Britain is pondering lender-of-last-resort facilities, which America intends to reserve for traditional banks. 译：英国正在考虑最后贷款人设施，而美国打算把这种设施保留给传统银行。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：考虑最后贷款人设施。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：ponder 是外刊常用动词，表示认真考虑；facility 在政策语境中是机制/工具，不是普通设施。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：ponder = think about carefully 仔细考虑；facility = institutional service or arrangement 制度性工具/机制；lender-of-last-resort = emergency central-bank support 最后贷款人支持。&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：facility 可指设施、便利、金融工具；这里指央行支持机制。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：正式、政策讨论语体。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：考虑最后贷款人支持机制。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Britain is pondering lender-of-last-resort facilities, which America intends to reserve for traditional banks.&lt;br&gt;译：英国正在考虑最后贷款人设施，而美国打算把这种设施保留给传统银行。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：ponder = 仔细考虑；facility 在金融政策中是“机制/工具”，不是普通建筑设施。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：翻译 facility 时要结合语境译为“机制/工具/安排”。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. The government is pondering new facilities for green investment. 译：政府正在考虑新的绿色投资支持工具。&lt;br&gt;2. Universities are pondering support facilities for stressed students. 译：大学正在考虑为压力大的学生提供支持机制。</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：说明英国和美国对稳定币央行支持态度不同。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：翻译 facility 时要结合金融语境译为“工具/机制/安排”。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：The government is pondering new facilities for green investment. 译：政府正在考虑新的绿色投资支持工具。&lt;br&gt;Universities are pondering support facilities for students under stress. 译：大学正在考虑为压力中的学生提供支持机制。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：公共治理作文可用：Governments should ponder support facilities for vulnerable groups before crises occur. 译：政府应在危机发生前考虑弱势群体支持机制。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Governments should ponder support facilities for vulnerable groups before crises occur. 译：政府应在危机发生前考虑弱势群体支持机制。</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -745,12 +745,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Tokenised bank deposits will be formidable competition. 译：代币化银行存款将成为强有力的竞争者。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：强有力的竞争者；强大竞争。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：formidable 是考研高频态度词，表示令人敬畏、难以对付。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：formidable = impressive and difficult to deal with 强大且难对付的；competition = rival or rivalry 竞争者/竞争。English: it is stronger than strong competition.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：formidable 可形容 opponent, challenge, task, barrier。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：正式、带压力感。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：强有力的竞争者；难以对付的竞争。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Tokenised bank deposits will be formidable competition.&lt;br&gt;译：代币化银行存款将成为强有力的竞争者。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：formidable 比 strong 更强，含“令人敬畏、难对付”。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：态度题中 formidable 表示强到不可忽视，不是 ordinary。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Online platforms have become formidable competition for traditional shops. 译：线上平台已成为传统商店的强大竞争者。&lt;br&gt;2. Climate change is a formidable challenge for every country. 译：气候变化是每个国家面临的严峻挑战。</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：结尾指出稳定币会面对来自代币化银行存款的竞争。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：态度题中 formidable 暗示 strong enough to matter，不是 ordinary。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Online platforms have become formidable competition for traditional shops. 译：线上平台已成为传统商店的强大竞争者。&lt;br&gt;Climate change is a formidable challenge for every country. 译：气候变化是每个国家面临的严峻挑战。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：作文可用：Lack of self-discipline can become a formidable barrier to personal growth. 译：缺乏自律可能成为个人成长的巨大障碍。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Lack of self-discipline can become a formidable barrier to personal growth. 译：缺乏自律可能成为个人成长的巨大障碍。</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -767,12 +767,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Digital innovations pose an awkward question to those in charge of the arrangement: how to make the system more efficient without making it any less safe? 译：数字创新给负责这套安排的人提出了一个棘手问题：如何提高效率而不降低安全性？&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：提出一个棘手问题。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：高价值写作句块，可引出矛盾、问题和论证中心。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：pose = raise/put forward 提出；awkward = difficult to handle 棘手的。English: pose a question is more formal than ask a question.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：pose 可指摆姿势，也可指造成/提出，如 pose a risk/problem/question。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：正式、有问题意识。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：提出一个棘手问题。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Digital innovations pose an awkward question to those in charge of the arrangement: how to make the system more efficient without making it any less safe?&lt;br&gt;译：数字创新给负责这套安排的人提出了一个棘手问题：如何提高效率而不降低安全性？&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：pose a question = 提出问题；awkward = 难处理的。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：冒号后常解释 question 的具体内容，是主旨定位点。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Automation poses an awkward question to workers. 译：自动化给劳动者提出了一个棘手问题。&lt;br&gt;2. Online education poses an awkward question to schools. 译：在线教育给学校提出了一个棘手问题。</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：引出本文中心矛盾：效率和安全如何兼得。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：阅读中后面的冒号常解释 question 的具体内容。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Automation poses an awkward question to workers: how to adapt without losing dignity. 译：自动化给劳动者提出了一个棘手问题：如何在适应变化的同时不失去尊严。&lt;br&gt;Online education poses an awkward question to schools: how to expand access without lowering quality. 译：在线教育给学校提出了一个棘手问题：如何扩大机会而不降低质量。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：作文核心模板：A poses an awkward question to B: how to do X without doing Y. 适配科技、教育、环境、职场。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：A poses an awkward question to B: how to do X without doing Y. 译：A 给 B 提出棘手问题：如何做 X 而不做 Y。</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -784,17 +784,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>cross-border payments on conventional rails</t>
+          <t>cross-border payments / conventional rails</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：They promise faster and cheaper cross-border payments than on conventional rails. 译：与传统支付轨道相比，它们承诺提供更快、更便宜的跨境支付。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：传统轨道上的跨境支付。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：cross-border 是经济生活高频；rails 是熟词僻义，指支付基础设施。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：cross-border = across national borders 跨境；payment = act of paying 支付；rail = infrastructure channel 基础通道。English: payment rails are the systems through which money moves.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：rail 本义铁轨；金融科技中是支付轨道/基础设施。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：正式中带技术隐喻。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：跨境支付 / 传统支付轨道。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：They promise faster and cheaper cross-border payments than on conventional rails.&lt;br&gt;译：与传统支付轨道相比，它们承诺提供更快、更便宜的跨境支付。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：rail 本义铁轨；支付语境中是“支付基础设施/通道”。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：熟词僻义题可能考 rails，不能译成真实铁路。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Small exporters need cheaper cross-border payments. 译：小出口商需要更便宜的跨境支付。&lt;br&gt;2. Digital platforms can improve old payment rails. 译：数字平台可以改进旧有支付基础设施。</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：说明稳定币可能改进跨境支付效率。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：熟词僻义题可能考 rails；不要译成真实铁路。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Small exporters need cheaper cross-border payments. 译：小出口商需要更便宜的跨境支付。&lt;br&gt;Digital platforms can improve old payment rails. 译：数字平台可以改进旧有支付基础设施。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：经济科技作文可用：Digital tools can reduce the cost of cross-border payments. 译：数字工具可以降低跨境支付成本。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Digital tools can reduce the cost of cross-border payments. 译：数字工具可以降低跨境支付成本。</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -811,12 +811,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Stablecoins account for a fair bit of illicit activity on blockchains. 译：稳定币在区块链上的非法活动中占有相当一部分。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：占相当一部分。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：account for 是高频熟词僻义，a fair bit of 是外刊模糊数量表达。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：account for = make up/represent 占比；fair bit = quite a lot 相当多。English: the phrase gives a cautious but meaningful quantity.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：account for 还可指解释原因，如 explain why；本文是占比。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：客观但带风险提示。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：占相当一部分。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Stablecoins account for a fair bit of illicit activity on blockchains.&lt;br&gt;译：稳定币在区块链上的非法活动中占有相当一部分。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：account for = 占比/解释；a fair bit of = 相当多。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：细节题看 account for 后面的宾语；别只记“解释”。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Transport accounts for a fair bit of urban pollution. 译：交通占城市污染的相当一部分。&lt;br&gt;2. Part-time jobs account for a fair bit of students' stress. 译：兼职工作占学生压力的相当一部分。</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：说明稳定币与非法活动有关联。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：细节题看 account for 后的宾语；原因题看 account for 是否作 explain。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Transport accounts for a fair bit of urban pollution. 译：交通占城市污染的相当一部分。&lt;br&gt;Part-time jobs account for a fair bit of students' stress. 译：兼职工作占学生压力的相当一部分。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：环境/教育作文可用：Household waste accounts for a fair bit of urban pollution. 译：生活垃圾占城市污染的相当一部分。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Household waste accounts for a fair bit of urban pollution. 译：生活垃圾占城市污染的相当一部分。</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -833,12 +833,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Stablecoins are a source of worry if a coin suffers a run. 译：如果某种稳定币遭遇挤兑，它也会成为一个令人担忧的来源。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：遭遇挤兑。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：run 是熟词僻义，金融中指大量持有人同时赎回。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：suffer = experience something bad 遭受；run = sudden mass withdrawal 挤兑。English: a run happens when confidence collapses and many holders rush to get cash.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：run 可指跑步、经营、运行、一段时间；bank run = 银行挤兑。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：负面、危机语境。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：遭遇挤兑。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Stablecoins are a source of worry if a coin suffers a run.&lt;br&gt;译：如果某种稳定币遭遇挤兑，它也会成为一个令人担忧的来源。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：run 在金融中不是跑步，而是集中取钱/赎回。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：熟词僻义题和翻译题高价值；bank run = 银行挤兑。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. A weak bank may suffer a run if depositors lose confidence. 译：如果储户失去信心，薄弱银行可能遭遇挤兑。&lt;br&gt;2. The fund sold assets quickly to prevent a run. 译：该基金迅速出售资产以防止挤兑。</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：指出稳定币可能引发挤兑风险。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：翻译题必须译为“挤兑”，不能译成“跑步”。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：A weak bank may suffer a run if depositors lose confidence. 译：如果储户失去信心，薄弱银行可能遭遇挤兑。&lt;br&gt;A platform can suffer a run of withdrawals after a security scandal. 译：安全丑闻后，平台可能遭遇集中提款。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：诚信作文可用 run on confidence：Once public trust collapses, even a strong system may suffer a crisis. 译：一旦公共信任崩塌，即使强大的体系也可能遭遇危机。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：不建议作文使用，语境较窄。</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -855,12 +855,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：America's GENIUS Act, which comes into effect next year, permits distributors to pay rewards. 译：美国即将于明年生效的《GENIUS 法案》允许分销商支付奖励。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：生效；开始实施。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：法律政策类高频固定搭配。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：come into = enter a state 进入某状态；effect = legal force/effective operation 效力。English: a law comes into effect when it starts to apply.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：effect 是名词“影响/效力”；affect 是动词“影响”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：正式、法律语体。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：生效；开始实施。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：America's GENIUS Act, which comes into effect next year, permits distributors to pay rewards.&lt;br&gt;译：美国即将于明年生效的《GENIUS 法案》允许分销商支付奖励。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：effect 是“效力/影响”；come into effect = 法规开始有效。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：法律政策类文章常替换为 take effect / become effective。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. The new school rule will come into effect next semester. 译：新校规将于下学期生效。&lt;br&gt;2. The environmental policy came into effect after months of debate. 译：经过数月辩论后，该环保政策开始实施。</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：介绍美国稳定币法律的时间和内容。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：同义替换：take effect, become effective, be implemented。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：The new school rule will come into effect next semester. 译：新校规将于下学期生效。&lt;br&gt;The environmental policy came into effect after months of debate. 译：经过数月辩论后，该环保政策开始实施。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：社会治理作文可用：Rules should come into effect only after careful public discussion. 译：规则应在充分公共讨论后实施。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Rules should come into effect only after careful public discussion. 译：规则应在充分公共讨论后实施。</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -877,12 +877,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Only a fraction of bank money is covered by such reserves. 译：银行货币只有一小部分由这类储备覆盖。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：一小部分。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：数量表达，常用于对比整体与部分。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：fraction = part of a whole 整体的一部分。English: a fraction of usually suggests a small share unless context says otherwise.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：fraction 数学中是分数；普通语境中是小部分。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：中性，但常带“少于预期”的暗示。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：一小部分。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Only a fraction of bank money is covered by such reserves.&lt;br&gt;译：银行货币只有一小部分由这类储备覆盖。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：fraction = 整体的一部分；a fraction of 通常暗示比例较小。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：长句翻译时注意 which 指代 bank money。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Only a fraction of students have access to high-quality rural education. 译：只有一小部分学生能获得高质量乡村教育。&lt;br&gt;2. A fraction of household waste can still cause serious pollution. 译：一小部分生活垃圾仍可能造成严重污染。</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Circle 老板用它对比稳定币全额储备与银行部分准备金。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：长句翻译时注意 which 指代 bank money。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Only a fraction of students have access to high-quality rural education. 译：只有一小部分学生能获得高质量乡村教育。&lt;br&gt;A fraction of household waste can still cause serious pollution. 译：一小部分生活垃圾仍可能造成严重污染。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：教育公平作文可用：Only a fraction of children should not enjoy most educational resources. 译：不应只有少数儿童享受大部分教育资源。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：Educational resources should not be enjoyed by only a fraction of children. 译：教育资源不应只由少数儿童享有。</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -899,12 +899,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Tokenised bank deposits, combining programmability with the backing and reputation of established institutions, will be formidable competition. 译：代币化银行存款将可编程性与成熟机构的支撑和声誉结合起来，会成为强有力的竞争者。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：代币化银行存款。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：金融科技主题词，理解其结构比背技术细节更重要。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：tokenise = turn into digital tokens 代币化；bank deposits = money held in bank accounts 银行存款。English: tokenised deposits are bank deposits represented in digital-token form.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：deposit 可指存款、押金、沉积物；本文是银行存款。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：正式、金融科技语体。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：代币化银行存款。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：Tokenised bank deposits, combining programmability with the backing and reputation of established institutions, will be formidable competition.&lt;br&gt;译：代币化银行存款将可编程性与成熟机构的支撑和声誉结合起来，会成为强有力的竞争者。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：tokenise = 转成数字代币；deposit 这里是“存款”。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：理解结构即可：它不是普通加密币，而是银行存款的数字代币形式。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. Tokenised bank deposits may make payments faster. 译：代币化银行存款可能让支付更快。&lt;br&gt;2. Digital certificates can tokenise ownership of cultural assets. 译：数字证书可以把文化资产所有权代币化。</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：结尾指出稳定币未来竞争者。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：阅读中注意它结合 programmability 与 established institutions，不是普通加密币。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：Tokenised bank deposits may make payments faster. 译：代币化银行存款可能让支付更快。&lt;br&gt;Digital certificates can tokenise ownership of cultural assets. 译：数字证书可以把文化资产所有权代币化。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：不建议作文使用，语境较窄。</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -921,12 +921,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：What matters most of all is that the great monetary confidence trick keeps working. 译：最重要的是，那场伟大的货币信任把戏必须继续运转。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：最重要的是……。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：主语从句 + 表语从句式强调句，作文结尾高价值。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：what matters = the thing that is important 重要的事情；most of all = above everything else 最重要。English: the structure foregrounds the core judgement.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：matter 可作名词“事情/物质”，动词“重要”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：总结性、强调性。</t>
+          <t>&lt;b&gt;核心意思&lt;/b&gt;：最重要的是……。&lt;br&gt;&lt;b&gt;原文句&lt;/b&gt;：What matters most of all is that the great monetary confidence trick keeps working.&lt;br&gt;译：最重要的是，那场伟大的货币信任把戏必须继续运转。&lt;br&gt;&lt;b&gt;怎么记&lt;/b&gt;：what matters = 重要的事情；that 后接完整句。&lt;br&gt;&lt;b&gt;怎么考&lt;/b&gt;：主旨题和结论题常围绕 what matters most 定位。&lt;br&gt;&lt;b&gt;真实例句&lt;/b&gt;：1. What matters most of all is that children learn to think independently. 译：最重要的是，孩子学会独立思考。&lt;br&gt;2. What matters most of all is that economic growth benefits ordinary people. 译：最重要的是，经济增长惠及普通人。</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：作者结尾把讨论升华为维护货币信任体系。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：主旨题和结论题常围绕 what matters most 定位。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先判断它在句中表达功能：定义、原因、风险、让步、对比还是结论；再看选项是否用同义替换偷换程度。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：常见同义替换包括 function, role, support, risk, regulate, effective, reliable；错误选项常把谨慎态度改成完全赞成或完全否定。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：What matters most of all is that children learn to think independently. 译：最重要的是，孩子学会独立思考。&lt;br&gt;What matters most of all is that economic growth benefits ordinary people. 译：最重要的是，经济增长惠及普通人。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：作文结尾模板：What matters most of all is that progress should serve human well-being. 译：最重要的是，进步应服务于人的福祉。</t>
+          <t>&lt;b&gt;作文可用&lt;/b&gt;：What matters most of all is that progress should serve human well-being. 译：最重要的是，进步应服务于人的福祉。</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>&lt;b&gt;适配话题&lt;/b&gt;：科技监管、教育科技、社会责任、公共治理。&lt;br&gt;&lt;b&gt;替换槽位&lt;/b&gt;：A = artificial intelligence / online education / digital platforms; B = policymakers / schools / companies; X = improve efficiency / expand access; Y = weakening fairness / harming privacy / reducing safety.&lt;br&gt;&lt;b&gt;多场景改写&lt;/b&gt;：1. Online education poses an awkward question to schools: how to expand access without lowering teaching quality. 译：在线教育给学校提出了一个棘手问题：如何扩大机会而不降低教学质量。&lt;br&gt;2. Fast economic growth poses an awkward question to governments: how to create wealth without damaging the environment. 译：快速经济增长给政府提出了一个棘手问题：如何创造财富而不破坏环境。&lt;br&gt;3. Digital platforms pose an awkward question to society: how to encourage innovation without sacrificing privacy. 译：数字平台给社会提出了一个棘手问题：如何鼓励创新而不牺牲隐私。&lt;br&gt;&lt;b&gt;常见错误&lt;/b&gt;：用 pose a question to sb，不写 pose sb a question；后面 how to...without... 很适合搭配。&lt;br&gt;&lt;b&gt;记忆抓手&lt;/b&gt;：pose = put forward; awkward = hard to handle.</t>
+          <t>&lt;b&gt;适配话题&lt;/b&gt;：科技监管、教育科技、社会责任、公共治理。&lt;br&gt;&lt;b&gt;替换槽位&lt;/b&gt;：A = artificial intelligence / online education / digital platforms; B = policymakers / schools / companies; X = improve efficiency / expand access; Y = weakening fairness / harming privacy / reducing safety.&lt;br&gt;&lt;b&gt;多场景改写&lt;/b&gt;：1. Online education poses an awkward question to schools: how to expand access without lowering teaching quality. 译：在线教育给学校提出了一个棘手问题：如何扩大机会而不降低教学质量。&lt;br&gt;2. Fast economic growth poses an awkward question to governments: how to create wealth without damaging the environment. 译：快速经济增长给政府提出了一个棘手问题：如何创造财富而不破坏环境。&lt;br&gt;3. Digital platforms pose an awkward question to society: how to encourage innovation without sacrificing privacy. 译：数字平台给社会提出了一个棘手问题：如何鼓励创新而不牺牲隐私。&lt;br&gt;&lt;b&gt;常见错误&lt;/b&gt;：用 pose a question to sb；后面 how to...without... 很适合接平衡型论证。&lt;br&gt;&lt;b&gt;记忆抓手&lt;/b&gt;：pose = put forward; awkward = hard to handle.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>&lt;b&gt;适配话题&lt;/b&gt;：公共服务、科技生活、教育公平、社会责任。&lt;br&gt;&lt;b&gt;替换槽位&lt;/b&gt;：A = public services / schools / digital platforms; efficient = accessible / affordable; safe = fair / reliable / accountable.&lt;br&gt;&lt;b&gt;多场景改写&lt;/b&gt;：1. Schools should make online learning more accessible without making it any less rigorous. 译：学校应让在线学习更易获得，同时不降低其严谨性。&lt;br&gt;2. Companies should make work more flexible without making it any less humane. 译：企业应让工作更灵活，同时不降低其人性化程度。&lt;br&gt;3. Cities should make transport faster without making it any less safe. 译：城市应让交通更快捷，同时不降低安全性。&lt;br&gt;&lt;b&gt;常见错误&lt;/b&gt;：any less 后接形容词，表示“一点也不更……/并不降低……”。&lt;br&gt;&lt;b&gt;记忆抓手&lt;/b&gt;：efficient + safe/fair 是考研作文高频平衡对。</t>
+          <t>&lt;b&gt;适配话题&lt;/b&gt;：公共服务、科技生活、教育公平、社会责任。&lt;br&gt;&lt;b&gt;替换槽位&lt;/b&gt;：A = public services / schools / digital platforms; efficient = accessible / affordable; safe = fair / reliable / accountable.&lt;br&gt;&lt;b&gt;多场景改写&lt;/b&gt;：1. Schools should make online learning more accessible without making it any less rigorous. 译：学校应让在线学习更易获得，同时不降低其严谨性。&lt;br&gt;2. Companies should make work more flexible without making it any less humane. 译：企业应让工作更灵活，同时不降低其人性化程度。&lt;br&gt;3. Cities should make transport faster without making it any less safe. 译：城市应让交通更快捷，同时不降低安全性。&lt;br&gt;&lt;b&gt;常见错误&lt;/b&gt;：any less 后接形容词，表示“不降低……”。&lt;br&gt;&lt;b&gt;记忆抓手&lt;/b&gt;：efficient + safe/fair 是作文高频平衡对。</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -992,7 +992,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>&lt;b&gt;适配话题&lt;/b&gt;：诚信、社会责任、职场伦理、环境保护。&lt;br&gt;&lt;b&gt;替换槽位&lt;/b&gt;：A = a promise / public trust / educational reform; B = concrete action / clear rules / sustained investment.&lt;br&gt;&lt;b&gt;多场景改写&lt;/b&gt;：1. Environmental protection should be backed by daily habits, not empty slogans. 译：环境保护应由日常习惯支撑，而不是空洞口号。&lt;br&gt;2. Educational fairness should be backed by sustained public investment. 译：教育公平应由持续的公共投入支撑。&lt;br&gt;3. Corporate integrity should be backed by transparent rules. 译：企业诚信应由透明规则支撑。&lt;br&gt;&lt;b&gt;常见错误&lt;/b&gt;：be backed by 是被动结构，不要漏掉 by；back 在这里不是“后背”。&lt;br&gt;&lt;b&gt;记忆抓手&lt;/b&gt;：back = support.</t>
+          <t>&lt;b&gt;适配话题&lt;/b&gt;：诚信、社会责任、职场伦理、环境保护。&lt;br&gt;&lt;b&gt;替换槽位&lt;/b&gt;：A = a promise / public trust / educational reform; B = concrete action / clear rules / sustained investment.&lt;br&gt;&lt;b&gt;多场景改写&lt;/b&gt;：1. Environmental protection should be backed by daily habits, not empty slogans. 译：环境保护应由日常习惯支撑，而不是空洞口号。&lt;br&gt;2. Educational fairness should be backed by sustained public investment. 译：教育公平应由持续的公共投入支撑。&lt;br&gt;3. Corporate integrity should be backed by transparent rules. 译：企业诚信应由透明规则支撑。&lt;br&gt;&lt;b&gt;常见错误&lt;/b&gt;：back 在这里不是“后背”，而是 support。&lt;br&gt;&lt;b&gt;记忆抓手&lt;/b&gt;：back = support.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>&lt;b&gt;适配话题&lt;/b&gt;：科技生活、公共服务、职场效率、教育数字化。&lt;br&gt;&lt;b&gt;替换槽位&lt;/b&gt;：A = digital tools / clear rules / online platforms; B = queue for hours / repeat paperwork / travel long distances.&lt;br&gt;&lt;b&gt;多场景改写&lt;/b&gt;：1. Online registration can obviate the need to wait in long lines. 译：在线注册可以免去长时间排队的需要。&lt;br&gt;2. Clear workplace rules can obviate the need for repeated negotiation. 译：明确的职场规则可以免去反复协商的需要。&lt;br&gt;3. Remote medical services can obviate the need to travel for basic consultations. 译：远程医疗服务可以免去基础咨询时长途奔波的需要。&lt;br&gt;&lt;b&gt;常见错误&lt;/b&gt;：obviate 是正式词，后面接名词或 the need to do；不要写 obviate to do。&lt;br&gt;&lt;b&gt;记忆抓手&lt;/b&gt;：obviate = remove the need.</t>
+          <t>&lt;b&gt;适配话题&lt;/b&gt;：科技生活、公共服务、职场效率、教育数字化。&lt;br&gt;&lt;b&gt;替换槽位&lt;/b&gt;：A = digital tools / clear rules / online platforms; B = queue for hours / repeat paperwork / travel long distances.&lt;br&gt;&lt;b&gt;多场景改写&lt;/b&gt;：1. Online registration can obviate the need to wait in long lines. 译：在线注册可以免去长时间排队的需要。&lt;br&gt;2. Clear workplace rules can obviate the need for repeated negotiation. 译：明确的职场规则可以免去反复协商的需要。&lt;br&gt;3. Remote medical services can obviate the need to travel for basic consultations. 译：远程医疗服务可以免去基础咨询时长途奔波的需要。&lt;br&gt;&lt;b&gt;常见错误&lt;/b&gt;：obviate 后接名词或 the need to do；不要写 obviate to do。&lt;br&gt;&lt;b&gt;记忆抓手&lt;/b&gt;：obviate = remove the need.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1036,7 +1036,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>&lt;b&gt;适配话题&lt;/b&gt;：科技、文化、教育、社会责任。&lt;br&gt;&lt;b&gt;替换槽位&lt;/b&gt;：A = technological changes / reforms / online trends; B = society / schools / young people; C = protect values / set priorities / act responsibly.&lt;br&gt;&lt;b&gt;多场景改写&lt;/b&gt;：1. Amid a flurry of education reforms, schools should protect students' curiosity. 译：在一连串教育改革中，学校应保护学生的好奇心。&lt;br&gt;2. Amid a flurry of online trends, young people should develop independent judgement. 译：在一连串网络潮流中，年轻人应培养独立判断。&lt;br&gt;3. Amid a flurry of environmental policies, citizens should take daily action. 译：在一连串环保政策中，公民应采取日常行动。&lt;br&gt;&lt;b&gt;常见错误&lt;/b&gt;：amid 后接名词短语；flurry 表“短时间密集出现”，不要译成普通 many。&lt;br&gt;&lt;b&gt;记忆抓手&lt;/b&gt;：amid = in the middle of; flurry = sudden burst.</t>
+          <t>&lt;b&gt;适配话题&lt;/b&gt;：科技、文化、教育、社会责任。&lt;br&gt;&lt;b&gt;替换槽位&lt;/b&gt;：A = technological changes / reforms / online trends; B = society / schools / young people; C = protect values / set priorities / act responsibly.&lt;br&gt;&lt;b&gt;多场景改写&lt;/b&gt;：1. Amid a flurry of education reforms, schools should protect students' curiosity. 译：在一连串教育改革中，学校应保护学生的好奇心。&lt;br&gt;2. Amid a flurry of online trends, young people should develop independent judgement. 译：在一连串网络潮流中，年轻人应培养独立判断。&lt;br&gt;3. Amid a flurry of environmental policies, citizens should take daily action. 译：在一连串环保政策中，公民应采取日常行动。&lt;br&gt;&lt;b&gt;常见错误&lt;/b&gt;：amid 后接名词短语；flurry 表“短时间密集出现”。&lt;br&gt;&lt;b&gt;记忆抓手&lt;/b&gt;：amid = in the middle of; flurry = sudden burst.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>&lt;b&gt;适配话题&lt;/b&gt;：科技、教育、健康、环境、社会责任、精神品质。&lt;br&gt;&lt;b&gt;替换槽位&lt;/b&gt;：progress = technology / education / economic growth; human well-being = fairness / health / dignity / public trust.&lt;br&gt;&lt;b&gt;多场景改写&lt;/b&gt;：1. What matters most of all is that education should help students become independent thinkers. 译：最重要的是，教育应帮助学生成为独立思考者。&lt;br&gt;2. What matters most of all is that economic growth should not damage the environment. 译：最重要的是，经济增长不应破坏环境。&lt;br&gt;3. What matters most of all is that technology should strengthen, not weaken, public trust. 译：最重要的是，技术应增强而不是削弱公共信任。&lt;br&gt;&lt;b&gt;常见错误&lt;/b&gt;：that 后必须接完整句；不要写 What matters most is to... 作为本卡主模板。&lt;br&gt;&lt;b&gt;记忆抓手&lt;/b&gt;：what matters = the key point.</t>
+          <t>&lt;b&gt;适配话题&lt;/b&gt;：科技、教育、健康、环境、社会责任、精神品质。&lt;br&gt;&lt;b&gt;替换槽位&lt;/b&gt;：progress = technology / education / economic growth; human well-being = fairness / health / dignity / public trust.&lt;br&gt;&lt;b&gt;多场景改写&lt;/b&gt;：1. What matters most of all is that education should help students become independent thinkers. 译：最重要的是，教育应帮助学生成为独立思考者。&lt;br&gt;2. What matters most of all is that economic growth should not damage the environment. 译：最重要的是，经济增长不应破坏环境。&lt;br&gt;3. What matters most of all is that technology should strengthen, not weaken, public trust. 译：最重要的是，技术应增强而不是削弱公共信任。&lt;br&gt;&lt;b&gt;常见错误&lt;/b&gt;：that 后必须接完整句。&lt;br&gt;&lt;b&gt;记忆抓手&lt;/b&gt;：what matters = the key point.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">

</xml_diff>